<commit_message>
Update BRDF _unc patch and cruise log
</commit_message>
<xml_diff>
--- a/Experiment_Cruise_Instrument_Radiometry_Field_Log.xlsx
+++ b/Experiment_Cruise_Instrument_Radiometry_Field_Log.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10720"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daurin/GitRepos/HyperCP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD160CA-28CE-4A48-9596-DF73E7415C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768EB23D-1D9F-6447-976B-D49CBDE7361B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="45760" yWindow="2000" windowWidth="34560" windowHeight="21560" xr2:uid="{334D9F36-0597-1A47-89E0-CF51DBBDBDB1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="39">
   <si>
     <t>lat</t>
   </si>
@@ -110,9 +110,6 @@
     <t>ship speed</t>
   </si>
   <si>
-    <t>(kts)</t>
-  </si>
-  <si>
     <t>solar disk</t>
   </si>
   <si>
@@ -149,14 +146,112 @@
     <t>(not req'd for autonomous systems when working properly, or if station number is in the name or ancillary SeaBASS file)</t>
   </si>
   <si>
-    <t>Experiment name (agreed upon for SeaBASS submission), Cruise name, ship/platform name, operator name. Set-up notes: height above water, ship hull color, etc., for autonomous systems include min/max azimuth settings, azimuth offset (usually 0, but confirm).</t>
+    <r>
+      <t>[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="0" tint="-0.249977111117893"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Experiment name (agreed upon for SeaBASS submission)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>], [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="0" tint="-0.249977111117893"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Cruise name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>], [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="0" tint="-0.249977111117893"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Ship/Platform name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>], [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="0" tint="-0.249977111117893"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Operator name</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>]. Set-up notes: [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="0" tint="-0.249977111117893"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>height above water, ship hull color, etc., for autonomous systems include min/max azimuth settings, azimuth offset (usually 0, but confirm).</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>]</t>
+    </r>
+  </si>
+  <si>
+    <t>(specify kts or m/s)</t>
+  </si>
+  <si>
+    <t>(Not required if obtained from autonmous observatories on ships/buoys.)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -180,6 +275,12 @@
       <b/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color theme="0" tint="-0.249977111117893"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -233,7 +334,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -249,6 +350,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -590,7 +694,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B1" s="7"/>
       <c r="C1" s="7"/>
@@ -668,17 +772,20 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
-      <c r="R4" s="1"/>
+      <c r="L4" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="8"/>
     </row>
     <row r="5" spans="1:20" ht="49" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>17</v>
@@ -720,16 +827,16 @@
         <v>13</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="S5" s="5" t="s">
         <v>15</v>
@@ -740,13 +847,13 @@
     </row>
     <row r="6" spans="1:20" s="1" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D6" s="3" t="s">
         <v>2</v>
@@ -757,17 +864,17 @@
       <c r="F6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>24</v>
+      <c r="G6" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>37</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J6" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>5</v>
@@ -788,10 +895,10 @@
         <v>7</v>
       </c>
       <c r="Q6" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R6" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="S6" s="3" t="s">
         <v>6</v>
@@ -801,8 +908,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:T3"/>
+    <mergeCell ref="L4:S4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>